<commit_message>
chore: 更新 Dashboard 数据 2026-10-15
</commit_message>
<xml_diff>
--- a/data-dashboard/public/data/美团数据.xlsx
+++ b/data-dashboard/public/data/美团数据.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D626"/>
+  <dimension ref="A1:D627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10450,6 +10450,22 @@
         <v>2648.99</v>
       </c>
     </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B627" t="n">
+        <v>1</v>
+      </c>
+      <c r="C627" t="n">
+        <v>363</v>
+      </c>
+      <c r="D627" t="n">
+        <v>2805.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>